<commit_message>
Perform backend security assessment, generate detailed vulnerability reports, and update scanner script
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/endpoint-inventory.xlsx
+++ b/Vulnerability Test Results/endpoint-inventory.xlsx
@@ -41,8 +41,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A8A"/>
-        <bgColor rgb="001E3A8A"/>
+        <fgColor rgb="001A365D"/>
+        <bgColor rgb="001A365D"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,16 +56,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00E2E8F0"/>
       </left>
       <right style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00E2E8F0"/>
       </right>
       <top style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00E2E8F0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00E2E8F0"/>
       </bottom>
     </border>
   </borders>
@@ -78,7 +78,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -485,12 +485,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>/register.php</t>
+          <t>/db_connect.php</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -505,19 +505,19 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>endo_backend_/register.php</t>
+          <t>endo_backend_/db_connect.php</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>/login.php</t>
+          <t>/get_patients.php</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -532,19 +532,19 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>endo_backend_/login.php</t>
+          <t>endo_backend_/get_patients.php</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>/get_patients.php</t>
+          <t>/login.php</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -559,7 +559,34 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>endo_backend_/get_patients.php</t>
+          <t>endo_backend_/login.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>/register.php</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Guest/Any</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>endo_backend_/register.php</t>
         </is>
       </c>
     </row>

</xml_diff>